<commit_message>
serial latency : default, CMD_VERSION 추가
</commit_message>
<xml_diff>
--- a/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_fw_release.xlsx
+++ b/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_fw_release.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD04P\LED_Module_Control_BD\XD04_LED_Module_Control_BD\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86034B57-7E51-433B-BC4E-E3F6C20FAE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7EC6AED-AE8B-430F-B1B4-E8C0DC006C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
+    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
   </bookViews>
   <sheets>
     <sheet name="fw release" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>Number</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -164,6 +164,22 @@
   </si>
   <si>
     <t xml:space="preserve">Screen for : CH Dependency, SCAN No., Line Delay </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"26. 06. 11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xdic_led_module_control_bd_release_260611.hex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xdic의 serial latency 설정 변경 : 60 -&gt; 200, CMD_VERSION 추가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Version Code</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -595,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5E52BB-E1D5-4646-A95E-7F5D1E996CD9}">
-  <dimension ref="B2:E12"/>
+  <dimension ref="B2:F13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.58203125" style="1" customWidth="1"/>
@@ -603,10 +619,11 @@
     <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="51.75" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="59" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.6640625" style="1"/>
+    <col min="6" max="6" width="10.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -619,8 +636,11 @@
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F2" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -633,8 +653,9 @@
       <c r="E3" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -647,8 +668,9 @@
       <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
@@ -659,8 +681,9 @@
         <v>9</v>
       </c>
       <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B6" s="3">
         <v>3</v>
       </c>
@@ -673,8 +696,9 @@
       <c r="E6" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -687,8 +711,9 @@
       <c r="E7" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -701,8 +726,9 @@
       <c r="E8" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B9" s="3">
         <v>6</v>
       </c>
@@ -715,8 +741,9 @@
       <c r="E9" s="4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B10" s="3">
         <v>7</v>
       </c>
@@ -729,8 +756,9 @@
       <c r="E10" s="4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B11" s="3">
         <v>8</v>
       </c>
@@ -743,8 +771,9 @@
       <c r="E11" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B12" s="3">
         <v>9</v>
       </c>
@@ -756,6 +785,24 @@
       </c>
       <c r="E12" s="4" t="s">
         <v>32</v>
+      </c>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="B13" s="3">
+        <v>10</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>